<commit_message>
feat(invoice-processing): generalize skill and remove courier fee category
- Desensitize template assets (receipt template, monthly summary, example)
- Generalize README and skill docs from xile-team specific to generic use
- Drop 快递费 (courier) category: scripts, SKILL.md, README, docx/xlsx templates
- Replace real names/companies/invoices in assets with generic placeholders
- Update example totals and doctests to match (1857.02 -> 1230.62)
- Remove stale AGENTS.md
</commit_message>
<xml_diff>
--- a/skills/invoice-processing/assets/月度汇总模版.xlsx
+++ b/skills/invoice-processing/assets/月度汇总模版.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D164"/>
+  <dimension ref="A1:D159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -476,7 +476,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>黄卉</t>
+          <t>张三</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>26378324211049524479</t>
+          <t>26370000000000000001</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -534,7 +534,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>26112000002498561776</t>
+          <t>26370000000000000002</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -549,14 +549,14 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>渔阳饭店住宿</t>
+          <t>酒店住宿</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>26317000002499183548</t>
+          <t>26370000000000000003</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -578,7 +578,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>26317000002499183549</t>
+          <t>26370000000000000004</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -600,7 +600,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>26317000002500075011</t>
+          <t>26370000000000000005</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -651,7 +651,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>26947000000098530588</t>
+          <t>26370000000000000006</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>26117000001003274848</t>
+          <t>26370000000000000007</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -695,7 +695,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>26947000000098530584</t>
+          <t>26370000000000000008</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -717,7 +717,7 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>曹英辰</t>
+          <t>李四</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>26112000002473428496</t>
+          <t>26370000000000000009</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -768,14 +768,14 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>办公用品 海创采购</t>
+          <t>办公用品 办公采购</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>26112000002796202501</t>
+          <t>26370000000000000010</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>26117000001007107561</t>
+          <t>26370000000000000011</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -819,7 +819,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>26112000002812608256</t>
+          <t>26370000000000000012</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -834,14 +834,14 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>办公用品 海创采购</t>
+          <t>办公用品 办公采购</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>26114000000056564536</t>
+          <t>26370000000000000013</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -863,7 +863,7 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>26117000001012652147</t>
+          <t>26370000000000000014</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -878,14 +878,14 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>办公用品 山姆采购</t>
+          <t>办公用品 商超采购</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>26117000001012652153</t>
+          <t>26370000000000000015</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>办公用品 山姆采购</t>
+          <t>办公用品 商超采购</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>26112000002425528156</t>
+          <t>26370000000000000016</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -951,14 +951,14 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>餐饮费用（和黄卉）</t>
+          <t>餐饮费用（和张三）</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>快递费（626.40元）</t>
+          <t>交通费（199.10元）</t>
         </is>
       </c>
     </row>
@@ -987,7 +987,7 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>26117000000982610843</t>
+          <t>26370000000000000020</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -997,63 +997,27 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>12.50</t>
+          <t>199.10</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>顺丰同城急送</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>26117000000998853625</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>7月7日</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>145.70</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>闪送配送费</t>
-        </is>
-      </c>
-    </row>
+          <t>滴滴打车</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>26117000001005294069</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>7月7日</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>468.20</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>顺丰快递费</t>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>王五</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>交通费（199.10元）</t>
+          <t>交通费（43.80元）</t>
         </is>
       </c>
     </row>
@@ -1082,17 +1046,17 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>26117000001007829300</t>
+          <t>26370000000000000021</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>7月7日</t>
+          <t>7月3日</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>199.10</t>
+          <t>43.80</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -1101,17 +1065,18 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39" ht="24" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>武佳鑫</t>
+          <t>赵六</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>交通费（43.80元）</t>
+          <t>交通费（205.00元）</t>
         </is>
       </c>
     </row>
@@ -1140,36 +1105,37 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>26117000000981265727</t>
+          <t>26370000000000000022</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>7月3日</t>
+          <t>7月10日</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>43.80</t>
+          <t>205.00</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>滴滴打车</t>
-        </is>
-      </c>
-    </row>
+          <t>滴滴打车 3笔</t>
+        </is>
+      </c>
+    </row>
+    <row r="43"/>
     <row r="44" ht="24" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>宋名言</t>
+          <t>孙七</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>交通费（205.00元）</t>
+          <t>差旅费（7921.00元）</t>
         </is>
       </c>
     </row>
@@ -1198,197 +1164,234 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>26117000001022177468</t>
+          <t>26370000000000000023</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>7月10日</t>
+          <t>3月15日</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>205.00</t>
+          <t>212.00</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>滴滴打车 3笔</t>
+          <t>高铁 北京西-太原</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000024</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>3月16日</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>195.00</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>高铁 太原-北京丰台</t>
         </is>
       </c>
     </row>
     <row r="49" ht="24" customHeight="1">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>刘芳</t>
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000025</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>4月22日</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>990.00</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>机票 北京-西安 HU7237 孙七</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>差旅费（7921.00元）</t>
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000026</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>4月22日</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>990.00</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>机票 北京-西安 HU7237 吴九</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>发票编号</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>总金额(元)</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>简要说明</t>
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000027</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>5月25日</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>1450.00</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>机票 北京-西安 CA1223 孙七</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>26119121152004638108</t>
+          <t>26370000000000000028</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>3月15日</t>
+          <t>5月25日</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>212.00</t>
+          <t>1450.00</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>高铁 北京西-太原</t>
+          <t>机票 北京-西安 CA1223 吴九</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>26149126447000463226</t>
+          <t>26370000000000000029</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>3月16日</t>
+          <t>6月12日</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>195.00</t>
+          <t>314.00</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>高铁 太原-北京丰台</t>
+          <t>酒店住宿 酒店</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>26468880111042460731</t>
+          <t>26370000000000000030</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>4月22日</t>
+          <t>6月12日</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>990.00</t>
+          <t>2320.00</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>机票 北京-西安 HU7237 刘芳</t>
+          <t>代订机票 西安-北京 CA1210 孙七 吴九</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>26468880111042460732</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>4月22日</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>990.00</t>
-        </is>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>机票 北京-西安 HU7237 范维肖</t>
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>交通费（1943.50元）</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>26118999111042462995</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>5月25日</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>1450.00</t>
-        </is>
-      </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>机票 北京-西安 CA1223 刘芳</t>
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>发票编号</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>总金额(元)</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>简要说明</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>26118999111042463020</t>
+          <t>26370000000000000031</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>5月25日</t>
+          <t>6月12日</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>1450.00</t>
+          <t>17.80</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>机票 北京-西安 CA1223 范维肖</t>
+          <t>滴滴打车 太原</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>26142000000845832961</t>
+          <t>26370000000000000032</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
@@ -1398,19 +1401,19 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>314.00</t>
+          <t>133.83</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>酒店住宿 亚朵酒店</t>
+          <t>高德打车 3笔</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>26317000002163183526</t>
+          <t>26370000000000000033</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
@@ -1420,484 +1423,501 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>2320.00</t>
+          <t>1791.87</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>代订机票 西安-北京 CA1210 刘芳 范维肖</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>交通费（1943.50元）</t>
-        </is>
-      </c>
-    </row>
+          <t>滴滴打车 多笔</t>
+        </is>
+      </c>
+    </row>
+    <row r="60"/>
     <row r="61">
-      <c r="A61" s="4" t="inlineStr">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>周八</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>差旅费（7469.89元）</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t>发票编号</t>
         </is>
       </c>
-      <c r="B61" s="4" t="inlineStr">
+      <c r="B63" s="4" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C63" s="4" t="inlineStr">
         <is>
           <t>总金额(元)</t>
         </is>
       </c>
-      <c r="D61" s="4" t="inlineStr">
+      <c r="D63" s="4" t="inlineStr">
         <is>
           <t>简要说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
-        <is>
-          <t>26147000000185967695</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="inlineStr">
-        <is>
-          <t>6月12日</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>17.80</t>
-        </is>
-      </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>滴滴打车 太原</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>26117000000848213299</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>6月12日</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>133.83</t>
-        </is>
-      </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>高德打车 3笔</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>26117000000849219087</t>
+          <t>26370000000000000034</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>6月12日</t>
+          <t>6月13日</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>1791.87</t>
+          <t>1060.00</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>滴滴打车 多笔</t>
+          <t>机票 北京-上海 CA1519 周八</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000035</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>6月13日</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>1060.00</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>机票 北京-上海 CA1501 吴九</t>
         </is>
       </c>
     </row>
     <row r="66" ht="24" customHeight="1">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>刘悦</t>
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000036</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>6月13日</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>2350.00</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>机票 上海-北京 CA1510 吴九</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>差旅费（7469.89元）</t>
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000037</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>6月14日</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>960.00</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>机票 上海-北京 CA1520 周八</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>发票编号</t>
-        </is>
-      </c>
-      <c r="B68" s="4" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>总金额(元)</t>
-        </is>
-      </c>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>简要说明</t>
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000038</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>6月15日</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>550.00</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>酒店住宿 酒店</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>26118999211049646270</t>
+          <t>26370000000000000039</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>6月13日</t>
+          <t>6月15日</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>1060.00</t>
+          <t>689.89</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>机票 北京-上海 CA1519 刘悦</t>
+          <t>代订住宿 吴九 酒店</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>26118999211049646272</t>
+          <t>26370000000000000040</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>6月13日</t>
+          <t>7月7日</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>1060.00</t>
+          <t>800.00</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>机票 北京-上海 CA1501 范维肖</t>
+          <t>代订机票 上海-北京</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="inlineStr">
-        <is>
-          <t>26118999211049646264</t>
-        </is>
-      </c>
-      <c r="B71" s="5" t="inlineStr">
-        <is>
-          <t>6月13日</t>
-        </is>
-      </c>
-      <c r="C71" s="5" t="inlineStr">
-        <is>
-          <t>2350.00</t>
-        </is>
-      </c>
-      <c r="D71" s="6" t="inlineStr">
-        <is>
-          <t>机票 上海-北京 CA1510 范维肖</t>
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>交通费（116.90元）</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t>26118999211049646268</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="inlineStr">
-        <is>
-          <t>6月14日</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>960.00</t>
-        </is>
-      </c>
-      <c r="D72" s="6" t="inlineStr">
-        <is>
-          <t>机票 上海-北京 CA1520 刘悦</t>
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>发票编号</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>总金额(元)</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>简要说明</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>26312000003747913486</t>
+          <t>26370000000000000041</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>6月15日</t>
+          <t>7月6日</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>550.00</t>
+          <t>31.10</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>酒店住宿 上海中航泊悦酒店</t>
+          <t>滴滴打车 上海</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>26317000002185852549</t>
+          <t>26370000000000000042</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>6月15日</t>
+          <t>7月6日</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>689.89</t>
+          <t>85.80</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>代订住宿 范维肖 上海中航虹桥机场泊悦酒店</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="5" t="inlineStr">
-        <is>
-          <t>26317000002508501998</t>
-        </is>
-      </c>
-      <c r="B75" s="5" t="inlineStr">
-        <is>
-          <t>7月7日</t>
-        </is>
-      </c>
-      <c r="C75" s="5" t="inlineStr">
-        <is>
-          <t>800.00</t>
-        </is>
-      </c>
-      <c r="D75" s="6" t="inlineStr">
-        <is>
-          <t>代订机票 上海-北京</t>
-        </is>
-      </c>
-    </row>
+          <t>滴滴打车 4笔</t>
+        </is>
+      </c>
+    </row>
+    <row r="75"/>
     <row r="76">
-      <c r="A76" s="3" t="inlineStr">
-        <is>
-          <t>交通费（116.90元）</t>
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>吴九</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="4" t="inlineStr">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>餐饮费（11398.20元）</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
         <is>
           <t>发票编号</t>
         </is>
       </c>
-      <c r="B77" s="4" t="inlineStr">
+      <c r="B78" s="4" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="C77" s="4" t="inlineStr">
+      <c r="C78" s="4" t="inlineStr">
         <is>
           <t>总金额(元)</t>
         </is>
       </c>
-      <c r="D77" s="4" t="inlineStr">
+      <c r="D78" s="4" t="inlineStr">
         <is>
           <t>简要说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="5" t="inlineStr">
-        <is>
-          <t>26317000002500126370</t>
-        </is>
-      </c>
-      <c r="B78" s="5" t="inlineStr">
-        <is>
-          <t>7月6日</t>
-        </is>
-      </c>
-      <c r="C78" s="5" t="inlineStr">
-        <is>
-          <t>31.10</t>
-        </is>
-      </c>
-      <c r="D78" s="6" t="inlineStr">
-        <is>
-          <t>滴滴打车 上海</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>26117000001002962139</t>
+          <t>26370000000000000043</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>7月6日</t>
+          <t>6月6日</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>85.80</t>
+          <t>43.00</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>滴滴打车 4笔</t>
+          <t>餐饮 餐厅</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000044</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>6月6日</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>60.00</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="81" ht="24" customHeight="1">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>范维肖</t>
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000045</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>6月8日</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>231.70</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="3" t="inlineStr">
-        <is>
-          <t>餐饮费（11398.20元）</t>
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000046</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>6月15日</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>292.00</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="4" t="inlineStr">
-        <is>
-          <t>发票编号</t>
-        </is>
-      </c>
-      <c r="B83" s="4" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>总金额(元)</t>
-        </is>
-      </c>
-      <c r="D83" s="4" t="inlineStr">
-        <is>
-          <t>简要说明</t>
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000047</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>6月16日</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>526.00</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>26112000002294932771</t>
+          <t>dzfp_26112000002510999926</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>6月6日</t>
+          <t>6月21日</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>43.00</t>
+          <t>400.00</t>
         </is>
       </c>
       <c r="D84" s="6" t="inlineStr">
         <is>
-          <t>餐饮 喜山</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>26112000002295074461</t>
+          <t>26370000000000000048</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>6月6日</t>
+          <t>6月25日</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>60.00</t>
+          <t>56.00</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>餐饮 喜山</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>26112000002315143861</t>
+          <t>26370000000000000049</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>6月8日</t>
+          <t>6月25日</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>231.70</t>
+          <t>662.80</t>
         </is>
       </c>
       <c r="D86" s="6" t="inlineStr">
         <is>
-          <t>餐饮 粉苏苏亮马桥店</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>26114000000047103076</t>
+          <t>26370000000000000050</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>6月15日</t>
+          <t>6月27日</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
@@ -1907,1572 +1927,1463 @@
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>餐饮 阿尔哲利亚</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>26112000002445325051</t>
+          <t>26370000000000000051</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>6月16日</t>
+          <t>6月30日</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>526.00</t>
+          <t>1498.00</t>
         </is>
       </c>
       <c r="D88" s="6" t="inlineStr">
         <is>
-          <t>餐饮 渔娘</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>dzfp_26112000002510999926</t>
+          <t>26370000000000000052</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>6月21日</t>
+          <t>7月1日</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>400.00</t>
+          <t>569.00</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>餐饮 盛春楼饭庄</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>26112000002589064591</t>
+          <t>26370000000000000053</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>6月25日</t>
+          <t>7月3日</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>56.00</t>
+          <t>310.00</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr">
         <is>
-          <t>餐饮 喜山</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>26112000002594003911</t>
+          <t>26370000000000000054</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>6月25日</t>
+          <t>7月3日</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>662.80</t>
+          <t>348.00</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>餐饮 院子味道</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>26114000000049912426</t>
+          <t>26370000000000000055</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>6月27日</t>
+          <t>7月4日</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>292.00</t>
+          <t>236.20</t>
         </is>
       </c>
       <c r="D92" s="6" t="inlineStr">
         <is>
-          <t>餐饮 阿尔哲利亚</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>26112000002676028876</t>
+          <t>26370000000000000056</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>6月30日</t>
+          <t>7月6日</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>1498.00</t>
+          <t>239.00</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>餐饮 亚洲大酒店</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>26112000002704357861</t>
+          <t>26370000000000000057</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>7月1日</t>
+          <t>7月10日</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>569.00</t>
+          <t>5000.00</t>
         </is>
       </c>
       <c r="D94" s="6" t="inlineStr">
         <is>
-          <t>餐饮 福丸屋福泉</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>26112000002743105741</t>
+          <t>26370000000000000058</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>7月3日</t>
+          <t>7月11日</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>310.00</t>
+          <t>125.90</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>餐饮 火烧火燎</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>26114000000052941451</t>
+          <t>26370000000000000059</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>7月3日</t>
+          <t>7月11日</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>348.00</t>
+          <t>508.60</t>
         </is>
       </c>
       <c r="D96" s="6" t="inlineStr">
         <is>
-          <t>餐饮 阿尔哲利亚</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="5" t="inlineStr">
-        <is>
-          <t>26112000002751933061</t>
-        </is>
-      </c>
-      <c r="B97" s="5" t="inlineStr">
-        <is>
-          <t>7月4日</t>
-        </is>
-      </c>
-      <c r="C97" s="5" t="inlineStr">
-        <is>
-          <t>236.20</t>
-        </is>
-      </c>
-      <c r="D97" s="6" t="inlineStr">
-        <is>
-          <t>餐饮 拓荒者</t>
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>办公费（29756.63元）</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="5" t="inlineStr">
-        <is>
-          <t>26132000002170516531</t>
-        </is>
-      </c>
-      <c r="B98" s="5" t="inlineStr">
-        <is>
-          <t>7月6日</t>
-        </is>
-      </c>
-      <c r="C98" s="5" t="inlineStr">
-        <is>
-          <t>239.00</t>
-        </is>
-      </c>
-      <c r="D98" s="6" t="inlineStr">
-        <is>
-          <t>餐饮 臻玺</t>
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>发票编号</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>总金额(元)</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>简要说明</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>26112000002841450001</t>
+          <t>26370000000000000060</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>7月10日</t>
+          <t>5月21日</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>5000.00</t>
+          <t>1491.00</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>餐饮 高奇</t>
+          <t>榻榻米 家居采购</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>26112000002855294206</t>
+          <t>26370000000000000061</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>7月11日</t>
+          <t>6月5日</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>125.90</t>
+          <t>206.80</t>
         </is>
       </c>
       <c r="D100" s="6" t="inlineStr">
         <is>
-          <t>餐饮 粉苏苏亮马桥店</t>
+          <t>焙烤食品 烘焙店</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>26112000002856187921</t>
+          <t>26370000000000000062</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>7月11日</t>
+          <t>6月7日</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>508.60</t>
+          <t>74.00</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>餐饮 胜利园</t>
+          <t>咖啡 咖啡店</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="3" t="inlineStr">
-        <is>
-          <t>办公费（29756.63元）</t>
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000063</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>6月8日</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>2234.40</t>
+        </is>
+      </c>
+      <c r="D102" s="6" t="inlineStr">
+        <is>
+          <t>饮品饮料 电商采购</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="4" t="inlineStr">
-        <is>
-          <t>发票编号</t>
-        </is>
-      </c>
-      <c r="B103" s="4" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
-      <c r="C103" s="4" t="inlineStr">
-        <is>
-          <t>总金额(元)</t>
-        </is>
-      </c>
-      <c r="D103" s="4" t="inlineStr">
-        <is>
-          <t>简要说明</t>
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>digital_26327000001064033426</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>6月9日</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>299.00</t>
+        </is>
+      </c>
+      <c r="D103" s="6" t="inlineStr">
+        <is>
+          <t>玩具乐器 电商采购</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>26932000000813710461</t>
+          <t>26370000000000000064</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>5月21日</t>
+          <t>6月11日</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>1491.00</t>
+          <t>28.00</t>
         </is>
       </c>
       <c r="D104" s="6" t="inlineStr">
         <is>
-          <t>榻榻米 家居采购</t>
+          <t>图书 电商采购</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>26957000000014822166</t>
+          <t>26370000000000000065</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>6月5日</t>
+          <t>6月17日</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>206.80</t>
+          <t>24.90</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>焙烤食品 美心</t>
+          <t>通讯配件 电商采购</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>26117000000541091598</t>
+          <t>26370000000000000066</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>6月7日</t>
+          <t>6月19日</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>74.00</t>
+          <t>42.80</t>
         </is>
       </c>
       <c r="D106" s="6" t="inlineStr">
         <is>
-          <t>咖啡 咖世家</t>
+          <t>数据线 配件店</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>26127000000289791921</t>
+          <t>26370000000000000067</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>6月8日</t>
+          <t>6月22日</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>2234.40</t>
+          <t>273.00</t>
         </is>
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>饮品饮料 京东采购</t>
+          <t>艺术品 电商采购</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>digital_26327000001064033426</t>
+          <t>26370000000000000068</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>6月9日</t>
+          <t>6月24日</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>299.00</t>
+          <t>37.00</t>
         </is>
       </c>
       <c r="D108" s="6" t="inlineStr">
         <is>
-          <t>玩具乐器 京东采购</t>
+          <t>咖啡 咖啡店</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>26117000000842644265</t>
+          <t>26370000000000000069</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>6月11日</t>
+          <t>6月24日</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>28.00</t>
+          <t>188.00</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>图书 京东采购</t>
+          <t>艺术品 电商采购</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>26117000000874789381</t>
+          <t>26370000000000000070</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>6月17日</t>
+          <t>6月29日</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>24.90</t>
+          <t>29.90</t>
         </is>
       </c>
       <c r="D110" s="6" t="inlineStr">
         <is>
-          <t>通讯配件 京东采购</t>
+          <t>饮品饮料 电商采购</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>26952000002563022506</t>
+          <t>26370000000000000071</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>6月19日</t>
+          <t>6月29日</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>42.80</t>
+          <t>47.61</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>数据线 绿联</t>
+          <t>饮品饮料 电商采购</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>26117000000916087017</t>
+          <t>26370000000000000072</t>
         </is>
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>6月22日</t>
+          <t>6月29日</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
-          <t>273.00</t>
+          <t>268.92</t>
         </is>
       </c>
       <c r="D112" s="6" t="inlineStr">
         <is>
-          <t>艺术品 京东采购</t>
+          <t>饮品饮料 电商采购</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>26112000002576861611</t>
+          <t>26370000000000000073</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>6月24日</t>
+          <t>6月29日</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>37.00</t>
+          <t>935.00</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>咖啡 拉比卡</t>
+          <t>日用品 电商采购</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>26117000000911570371</t>
+          <t>5609470405</t>
         </is>
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>6月24日</t>
+          <t>6月30日</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>188.00</t>
+          <t>48.83</t>
         </is>
       </c>
       <c r="D114" s="6" t="inlineStr">
         <is>
-          <t>艺术品 京东采购</t>
+          <t>软件订阅费 (SGD)</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>26137000000321153896</t>
+          <t>26370000000000000074</t>
         </is>
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>6月29日</t>
+          <t>7月1日</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>29.90</t>
+          <t>20000.00</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>饮品饮料 京东采购</t>
+          <t>云服务费</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>26137000000321648815</t>
+          <t>26370000000000000075</t>
         </is>
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>6月29日</t>
+          <t>7月5日</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>47.61</t>
+          <t>169.31</t>
         </is>
       </c>
       <c r="D116" s="6" t="inlineStr">
         <is>
-          <t>饮品饮料 京东采购</t>
+          <t>水果 采购</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>26137000000321648817</t>
+          <t>26370000000000000076</t>
         </is>
       </c>
       <c r="B117" s="5" t="inlineStr">
         <is>
-          <t>6月29日</t>
+          <t>7月7日</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>268.92</t>
+          <t>440.00</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>饮品饮料 京东采购</t>
+          <t>咖啡 咖啡店</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>26117000000950091005</t>
+          <t>26370000000000000077</t>
         </is>
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>6月29日</t>
+          <t>7月8日</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>935.00</t>
+          <t>139.00</t>
         </is>
       </c>
       <c r="D118" s="6" t="inlineStr">
         <is>
-          <t>日用品 京东采购</t>
+          <t>车载冰箱杯架</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>5609470405</t>
+          <t>26370000000000000078</t>
         </is>
       </c>
       <c r="B119" s="5" t="inlineStr">
         <is>
-          <t>6月30日</t>
+          <t>7月10日</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>48.83</t>
+          <t>1211.80</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>Google Workspace 订阅费 (SGD)</t>
+          <t>饮品饮料 电商采购</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>26117000000969931115</t>
+          <t>26370000000000000079</t>
         </is>
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>7月1日</t>
+          <t>7月10日</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>20000.00</t>
+          <t>1567.36</t>
         </is>
       </c>
       <c r="D120" s="6" t="inlineStr">
         <is>
-          <t>腾讯云服务费</t>
+          <t>艺术品 电商采购</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="5" t="inlineStr">
-        <is>
-          <t>26117000000973431531</t>
-        </is>
-      </c>
-      <c r="B121" s="5" t="inlineStr">
-        <is>
-          <t>7月5日</t>
-        </is>
-      </c>
-      <c r="C121" s="5" t="inlineStr">
-        <is>
-          <t>169.31</t>
-        </is>
-      </c>
-      <c r="D121" s="6" t="inlineStr">
-        <is>
-          <t>水果 采购</t>
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>替票（客户公司等）（100378.00元）</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="5" t="inlineStr">
-        <is>
-          <t>26117000000989201954</t>
-        </is>
-      </c>
-      <c r="B122" s="5" t="inlineStr">
-        <is>
-          <t>7月7日</t>
-        </is>
-      </c>
-      <c r="C122" s="5" t="inlineStr">
-        <is>
-          <t>440.00</t>
-        </is>
-      </c>
-      <c r="D122" s="6" t="inlineStr">
-        <is>
-          <t>咖啡 星巴克</t>
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t>发票编号</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>总金额(元)</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>简要说明</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>26112000002800646461</t>
+          <t>26370000000000000080</t>
         </is>
       </c>
       <c r="B123" s="5" t="inlineStr">
         <is>
-          <t>7月8日</t>
+          <t>6月23日</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>139.00</t>
+          <t>18350.00</t>
         </is>
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>车载冰箱杯架</t>
+          <t>替票 品牌男式T恤</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>26117000001024465407</t>
+          <t>26370000000000000081</t>
         </is>
       </c>
       <c r="B124" s="5" t="inlineStr">
         <is>
-          <t>7月10日</t>
+          <t>6月27日</t>
         </is>
       </c>
       <c r="C124" s="5" t="inlineStr">
         <is>
-          <t>1211.80</t>
+          <t>22600.00</t>
         </is>
       </c>
       <c r="D124" s="6" t="inlineStr">
         <is>
-          <t>饮品饮料 京东采购</t>
+          <t>替票 品牌女式半身裙</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>26117000001024465436</t>
+          <t>26370000000000000082</t>
         </is>
       </c>
       <c r="B125" s="5" t="inlineStr">
         <is>
-          <t>7月10日</t>
+          <t>7月7日</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>1567.36</t>
+          <t>2150.00</t>
         </is>
       </c>
       <c r="D125" s="6" t="inlineStr">
         <is>
-          <t>艺术品 京东采购</t>
+          <t>替票 美容仪</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="3" t="inlineStr">
-        <is>
-          <t>替票（南京乐擎等）（100378.00元）</t>
+      <c r="A126" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000083</t>
+        </is>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>7月8日</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>11500.00</t>
+        </is>
+      </c>
+      <c r="D126" s="6" t="inlineStr">
+        <is>
+          <t>替票 代订机票</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="4" t="inlineStr">
-        <is>
-          <t>发票编号</t>
-        </is>
-      </c>
-      <c r="B127" s="4" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
-      <c r="C127" s="4" t="inlineStr">
-        <is>
-          <t>总金额(元)</t>
-        </is>
-      </c>
-      <c r="D127" s="4" t="inlineStr">
-        <is>
-          <t>简要说明</t>
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000084</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>7月8日</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>19678.00</t>
+        </is>
+      </c>
+      <c r="D127" s="6" t="inlineStr">
+        <is>
+          <t>替票 代订机票</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
-          <t>26112000002549149516</t>
+          <t>26370000000000000085</t>
         </is>
       </c>
       <c r="B128" s="5" t="inlineStr">
         <is>
-          <t>6月23日</t>
+          <t>7月11日</t>
         </is>
       </c>
       <c r="C128" s="5" t="inlineStr">
         <is>
-          <t>18350.00</t>
+          <t>26100.00</t>
         </is>
       </c>
       <c r="D128" s="6" t="inlineStr">
         <is>
-          <t>替票 LV男式T恤</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="5" t="inlineStr">
-        <is>
-          <t>26112000002624594656</t>
-        </is>
-      </c>
-      <c r="B129" s="5" t="inlineStr">
-        <is>
-          <t>6月27日</t>
-        </is>
-      </c>
-      <c r="C129" s="5" t="inlineStr">
-        <is>
-          <t>22600.00</t>
-        </is>
-      </c>
-      <c r="D129" s="6" t="inlineStr">
-        <is>
-          <t>替票 LV女式半身裙</t>
-        </is>
-      </c>
-    </row>
+          <t>替票 品牌背提包</t>
+        </is>
+      </c>
+    </row>
+    <row r="129"/>
     <row r="130">
-      <c r="A130" s="5" t="inlineStr">
-        <is>
-          <t>26442000007714543726</t>
-        </is>
-      </c>
-      <c r="B130" s="5" t="inlineStr">
-        <is>
-          <t>7月7日</t>
-        </is>
-      </c>
-      <c r="C130" s="5" t="inlineStr">
-        <is>
-          <t>2150.00</t>
-        </is>
-      </c>
-      <c r="D130" s="6" t="inlineStr">
-        <is>
-          <t>替票 美容仪</t>
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>郑十</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="5" t="inlineStr">
-        <is>
-          <t>26512000002898457276</t>
-        </is>
-      </c>
-      <c r="B131" s="5" t="inlineStr">
-        <is>
-          <t>7月8日</t>
-        </is>
-      </c>
-      <c r="C131" s="5" t="inlineStr">
-        <is>
-          <t>11500.00</t>
-        </is>
-      </c>
-      <c r="D131" s="6" t="inlineStr">
-        <is>
-          <t>替票 代订机票</t>
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>餐饮费（3384.54元）</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="5" t="inlineStr">
-        <is>
-          <t>26337000000643706482</t>
-        </is>
-      </c>
-      <c r="B132" s="5" t="inlineStr">
-        <is>
-          <t>7月8日</t>
-        </is>
-      </c>
-      <c r="C132" s="5" t="inlineStr">
-        <is>
-          <t>19678.00</t>
-        </is>
-      </c>
-      <c r="D132" s="6" t="inlineStr">
-        <is>
-          <t>替票 代订机票</t>
+      <c r="A132" s="4" t="inlineStr">
+        <is>
+          <t>发票编号</t>
+        </is>
+      </c>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="C132" s="4" t="inlineStr">
+        <is>
+          <t>总金额(元)</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>简要说明</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t>26112000002856781036</t>
+          <t>26370000000000000086</t>
         </is>
       </c>
       <c r="B133" s="5" t="inlineStr">
         <is>
-          <t>7月11日</t>
+          <t>6月4日</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>26100.00</t>
+          <t>195.00</t>
         </is>
       </c>
       <c r="D133" s="6" t="inlineStr">
         <is>
-          <t>替票 LV背提包</t>
+          <t>餐饮 餐厅</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000087</t>
+        </is>
+      </c>
+      <c r="B134" s="5" t="inlineStr">
+        <is>
+          <t>6月4日</t>
+        </is>
+      </c>
+      <c r="C134" s="5" t="inlineStr">
+        <is>
+          <t>273.60</t>
+        </is>
+      </c>
+      <c r="D134" s="6" t="inlineStr">
+        <is>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="135" ht="24" customHeight="1">
-      <c r="A135" s="2" t="inlineStr">
-        <is>
-          <t>曹昱</t>
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000088</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>6月11日</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>201.30</t>
+        </is>
+      </c>
+      <c r="D135" s="6" t="inlineStr">
+        <is>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="3" t="inlineStr">
-        <is>
-          <t>餐饮费（3384.54元）</t>
+      <c r="A136" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000089</t>
+        </is>
+      </c>
+      <c r="B136" s="5" t="inlineStr">
+        <is>
+          <t>6月12日</t>
+        </is>
+      </c>
+      <c r="C136" s="5" t="inlineStr">
+        <is>
+          <t>88.00</t>
+        </is>
+      </c>
+      <c r="D136" s="6" t="inlineStr">
+        <is>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="4" t="inlineStr">
-        <is>
-          <t>发票编号</t>
-        </is>
-      </c>
-      <c r="B137" s="4" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
-      <c r="C137" s="4" t="inlineStr">
-        <is>
-          <t>总金额(元)</t>
-        </is>
-      </c>
-      <c r="D137" s="4" t="inlineStr">
-        <is>
-          <t>简要说明</t>
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>26370000000000000090</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>6月12日</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>1061.00</t>
+        </is>
+      </c>
+      <c r="D137" s="6" t="inlineStr">
+        <is>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
         <is>
-          <t>26112000002268959731</t>
+          <t>26370000000000000091</t>
         </is>
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>6月4日</t>
+          <t>6月29日</t>
         </is>
       </c>
       <c r="C138" s="5" t="inlineStr">
         <is>
-          <t>195.00</t>
+          <t>220.00</t>
         </is>
       </c>
       <c r="D138" s="6" t="inlineStr">
         <is>
-          <t>餐饮 超级浅也</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="5" t="inlineStr">
         <is>
-          <t>26112000002268960631</t>
+          <t>26370000000000000092</t>
         </is>
       </c>
       <c r="B139" s="5" t="inlineStr">
         <is>
-          <t>6月4日</t>
+          <t>6月29日</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>273.60</t>
+          <t>369.00</t>
         </is>
       </c>
       <c r="D139" s="6" t="inlineStr">
         <is>
-          <t>餐饮 苏小牛</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
         <is>
-          <t>26112000002381369506</t>
+          <t>26370000000000000093</t>
         </is>
       </c>
       <c r="B140" s="5" t="inlineStr">
         <is>
-          <t>6月11日</t>
+          <t>7月7日</t>
         </is>
       </c>
       <c r="C140" s="5" t="inlineStr">
         <is>
-          <t>201.30</t>
+          <t>82.06</t>
         </is>
       </c>
       <c r="D140" s="6" t="inlineStr">
         <is>
-          <t>餐饮 苏小牛</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="5" t="inlineStr">
         <is>
-          <t>26112000002390874181</t>
+          <t>26370000000000000094</t>
         </is>
       </c>
       <c r="B141" s="5" t="inlineStr">
         <is>
-          <t>6月12日</t>
+          <t>7月7日</t>
         </is>
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>88.00</t>
+          <t>87.08</t>
         </is>
       </c>
       <c r="D141" s="6" t="inlineStr">
         <is>
-          <t>餐饮 老乡鸡</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
         <is>
-          <t>26112000002398428271</t>
+          <t>26370000000000000095</t>
         </is>
       </c>
       <c r="B142" s="5" t="inlineStr">
         <is>
-          <t>6月12日</t>
+          <t>7月7日</t>
         </is>
       </c>
       <c r="C142" s="5" t="inlineStr">
         <is>
-          <t>1061.00</t>
+          <t>152.00</t>
         </is>
       </c>
       <c r="D142" s="6" t="inlineStr">
         <is>
-          <t>餐饮 湖小龙金棕榈</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="5" t="inlineStr">
         <is>
-          <t>26112000002649123826</t>
+          <t>26370000000000000096</t>
         </is>
       </c>
       <c r="B143" s="5" t="inlineStr">
         <is>
-          <t>6月29日</t>
+          <t>7月7日</t>
         </is>
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>220.00</t>
+          <t>332.20</t>
         </is>
       </c>
       <c r="D143" s="6" t="inlineStr">
         <is>
-          <t>餐饮 波兹</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="5" t="inlineStr">
         <is>
-          <t>26112000002662084966</t>
+          <t>26370000000000000097</t>
         </is>
       </c>
       <c r="B144" s="5" t="inlineStr">
         <is>
-          <t>6月29日</t>
+          <t>7月8日</t>
         </is>
       </c>
       <c r="C144" s="5" t="inlineStr">
         <is>
-          <t>369.00</t>
+          <t>202.80</t>
         </is>
       </c>
       <c r="D144" s="6" t="inlineStr">
         <is>
-          <t>餐饮 曾何适</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="5" t="inlineStr">
         <is>
-          <t>26114000000056382916</t>
+          <t>26370000000000000098</t>
         </is>
       </c>
       <c r="B145" s="5" t="inlineStr">
         <is>
-          <t>7月7日</t>
+          <t>7月9日</t>
         </is>
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>82.06</t>
+          <t>120.50</t>
         </is>
       </c>
       <c r="D145" s="6" t="inlineStr">
         <is>
-          <t>餐饮 养个好胃</t>
+          <t>餐饮 餐厅</t>
         </is>
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="5" t="inlineStr">
-        <is>
-          <t>26114000000055781416</t>
-        </is>
-      </c>
-      <c r="B146" s="5" t="inlineStr">
-        <is>
-          <t>7月7日</t>
-        </is>
-      </c>
-      <c r="C146" s="5" t="inlineStr">
-        <is>
-          <t>87.08</t>
-        </is>
-      </c>
-      <c r="D146" s="6" t="inlineStr">
-        <is>
-          <t>餐饮 养个好胃</t>
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>办公费（27772.08元）</t>
         </is>
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="5" t="inlineStr">
-        <is>
-          <t>26117000001008076828</t>
-        </is>
-      </c>
-      <c r="B147" s="5" t="inlineStr">
-        <is>
-          <t>7月7日</t>
-        </is>
-      </c>
-      <c r="C147" s="5" t="inlineStr">
-        <is>
-          <t>152.00</t>
-        </is>
-      </c>
-      <c r="D147" s="6" t="inlineStr">
-        <is>
-          <t>餐饮 海鸿达</t>
+      <c r="A147" s="4" t="inlineStr">
+        <is>
+          <t>发票编号</t>
+        </is>
+      </c>
+      <c r="B147" s="4" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="C147" s="4" t="inlineStr">
+        <is>
+          <t>总金额(元)</t>
+        </is>
+      </c>
+      <c r="D147" s="4" t="inlineStr">
+        <is>
+          <t>简要说明</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="5" t="inlineStr">
         <is>
-          <t>26112000002797666756</t>
+          <t>26370000000000000099</t>
         </is>
       </c>
       <c r="B148" s="5" t="inlineStr">
         <is>
-          <t>7月7日</t>
+          <t>6月14日</t>
         </is>
       </c>
       <c r="C148" s="5" t="inlineStr">
         <is>
-          <t>332.20</t>
+          <t>1024.00</t>
         </is>
       </c>
       <c r="D148" s="6" t="inlineStr">
         <is>
-          <t>餐饮 红红的店</t>
+          <t>保险柜 办公采购</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="5" t="inlineStr">
         <is>
-          <t>26112000002810983456</t>
+          <t>263700000000000000100</t>
         </is>
       </c>
       <c r="B149" s="5" t="inlineStr">
         <is>
-          <t>7月8日</t>
+          <t>7月7日</t>
         </is>
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>202.80</t>
+          <t>3350.08</t>
         </is>
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>餐饮 中食京六</t>
+          <t>平板电脑+触控笔</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="5" t="inlineStr">
         <is>
-          <t>26112000002821745446</t>
+          <t>263700000000000000101</t>
         </is>
       </c>
       <c r="B150" s="5" t="inlineStr">
         <is>
-          <t>7月9日</t>
+          <t>7月7日</t>
         </is>
       </c>
       <c r="C150" s="5" t="inlineStr">
         <is>
-          <t>120.50</t>
+          <t>3398.00</t>
         </is>
       </c>
       <c r="D150" s="6" t="inlineStr">
         <is>
-          <t>餐饮 林子豪</t>
+          <t>平板电脑+触控笔</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="3" t="inlineStr">
-        <is>
-          <t>办公费（27772.08元）</t>
+      <c r="A151" s="5" t="inlineStr">
+        <is>
+          <t>263700000000000000102</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>7月8日</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>20000.00</t>
+        </is>
+      </c>
+      <c r="D151" s="6" t="inlineStr">
+        <is>
+          <t>云服务费</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="4" t="inlineStr">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>差旅费（420.40元）</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="4" t="inlineStr">
         <is>
           <t>发票编号</t>
         </is>
       </c>
-      <c r="B152" s="4" t="inlineStr">
+      <c r="B153" s="4" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="C152" s="4" t="inlineStr">
+      <c r="C153" s="4" t="inlineStr">
         <is>
           <t>总金额(元)</t>
         </is>
       </c>
-      <c r="D152" s="4" t="inlineStr">
+      <c r="D153" s="4" t="inlineStr">
         <is>
           <t>简要说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="5" t="inlineStr">
-        <is>
-          <t>26132000001853927371</t>
-        </is>
-      </c>
-      <c r="B153" s="5" t="inlineStr">
-        <is>
-          <t>6月14日</t>
-        </is>
-      </c>
-      <c r="C153" s="5" t="inlineStr">
-        <is>
-          <t>1024.00</t>
-        </is>
-      </c>
-      <c r="D153" s="6" t="inlineStr">
-        <is>
-          <t>保险柜 办公采购</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="5" t="inlineStr">
         <is>
-          <t>26957000000184624223</t>
+          <t>263700000000000000103</t>
         </is>
       </c>
       <c r="B154" s="5" t="inlineStr">
         <is>
+          <t>6月24日</t>
+        </is>
+      </c>
+      <c r="C154" s="5" t="inlineStr">
+        <is>
+          <t>420.40</t>
+        </is>
+      </c>
+      <c r="D154" s="6" t="inlineStr">
+        <is>
+          <t>代订住宿 酒店</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>替票（1361.80元）</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="4" t="inlineStr">
+        <is>
+          <t>发票编号</t>
+        </is>
+      </c>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="C156" s="4" t="inlineStr">
+        <is>
+          <t>总金额(元)</t>
+        </is>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>简要说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>263700000000000000104</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>6月2日</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>799.00</t>
+        </is>
+      </c>
+      <c r="D157" s="6" t="inlineStr">
+        <is>
+          <t>替票 电器采购</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="5" t="inlineStr">
+        <is>
+          <t>263700000000000000105</t>
+        </is>
+      </c>
+      <c r="B158" s="5" t="inlineStr">
+        <is>
           <t>7月7日</t>
         </is>
       </c>
-      <c r="C154" s="5" t="inlineStr">
-        <is>
-          <t>3350.08</t>
-        </is>
-      </c>
-      <c r="D154" s="6" t="inlineStr">
-        <is>
-          <t>小米平板+触控笔</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="5" t="inlineStr">
-        <is>
-          <t>26957000000184624214</t>
-        </is>
-      </c>
-      <c r="B155" s="5" t="inlineStr">
-        <is>
-          <t>7月7日</t>
-        </is>
-      </c>
-      <c r="C155" s="5" t="inlineStr">
-        <is>
-          <t>3398.00</t>
-        </is>
-      </c>
-      <c r="D155" s="6" t="inlineStr">
-        <is>
-          <t>小米平板+触控笔</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="5" t="inlineStr">
-        <is>
-          <t>26117000001007471146</t>
-        </is>
-      </c>
-      <c r="B156" s="5" t="inlineStr">
-        <is>
-          <t>7月8日</t>
-        </is>
-      </c>
-      <c r="C156" s="5" t="inlineStr">
-        <is>
-          <t>20000.00</t>
-        </is>
-      </c>
-      <c r="D156" s="6" t="inlineStr">
-        <is>
-          <t>腾讯云服务费</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="3" t="inlineStr">
-        <is>
-          <t>差旅费（420.40元）</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="4" t="inlineStr">
-        <is>
-          <t>发票编号</t>
-        </is>
-      </c>
-      <c r="B158" s="4" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
-      <c r="C158" s="4" t="inlineStr">
-        <is>
-          <t>总金额(元)</t>
-        </is>
-      </c>
-      <c r="D158" s="4" t="inlineStr">
-        <is>
-          <t>简要说明</t>
+      <c r="C158" s="5" t="inlineStr">
+        <is>
+          <t>194.00</t>
+        </is>
+      </c>
+      <c r="D158" s="6" t="inlineStr">
+        <is>
+          <t>替票 水果</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="5" t="inlineStr">
         <is>
-          <t>26317000002272762017</t>
+          <t>263700000000000000106</t>
         </is>
       </c>
       <c r="B159" s="5" t="inlineStr">
         <is>
-          <t>6月24日</t>
+          <t>7月7日</t>
         </is>
       </c>
       <c r="C159" s="5" t="inlineStr">
         <is>
-          <t>420.40</t>
+          <t>368.80</t>
         </is>
       </c>
       <c r="D159" s="6" t="inlineStr">
-        <is>
-          <t>代订住宿 酒店</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="3" t="inlineStr">
-        <is>
-          <t>替票（1361.80元）</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="4" t="inlineStr">
-        <is>
-          <t>发票编号</t>
-        </is>
-      </c>
-      <c r="B161" s="4" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
-      <c r="C161" s="4" t="inlineStr">
-        <is>
-          <t>总金额(元)</t>
-        </is>
-      </c>
-      <c r="D161" s="4" t="inlineStr">
-        <is>
-          <t>简要说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="5" t="inlineStr">
-        <is>
-          <t>26117000000790878194</t>
-        </is>
-      </c>
-      <c r="B162" s="5" t="inlineStr">
-        <is>
-          <t>6月2日</t>
-        </is>
-      </c>
-      <c r="C162" s="5" t="inlineStr">
-        <is>
-          <t>799.00</t>
-        </is>
-      </c>
-      <c r="D162" s="6" t="inlineStr">
-        <is>
-          <t>替票 京东电器</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="5" t="inlineStr">
-        <is>
-          <t>26112000002798034601</t>
-        </is>
-      </c>
-      <c r="B163" s="5" t="inlineStr">
-        <is>
-          <t>7月7日</t>
-        </is>
-      </c>
-      <c r="C163" s="5" t="inlineStr">
-        <is>
-          <t>194.00</t>
-        </is>
-      </c>
-      <c r="D163" s="6" t="inlineStr">
-        <is>
-          <t>替票 水果</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="5" t="inlineStr">
-        <is>
-          <t>26112000002798911231</t>
-        </is>
-      </c>
-      <c r="B164" s="5" t="inlineStr">
-        <is>
-          <t>7月7日</t>
-        </is>
-      </c>
-      <c r="C164" s="5" t="inlineStr">
-        <is>
-          <t>368.80</t>
-        </is>
-      </c>
-      <c r="D164" s="6" t="inlineStr">
         <is>
           <t>替票 水果</t>
         </is>

</xml_diff>